<commit_message>
new figs, fixing data processing for tables
</commit_message>
<xml_diff>
--- a/output/tables/B25_Table1_publication_format.xlsx
+++ b/output/tables/B25_Table1_publication_format.xlsx
@@ -1,21 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10817"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/elizabeth/Documents/GitHub/ice-sheet-sej-2025/output/tables/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ABBEB09-2B6D-E840-9F5A-FFE00EFAC032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="760" windowWidth="25440" windowHeight="18640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Table 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -607,8 +601,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -662,8 +656,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -677,39 +674,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -747,7 +724,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -781,7 +758,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -816,10 +792,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -992,792 +967,750 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:M23"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="24.6640625" customWidth="1"/>
-    <col min="2" max="5" width="14.6640625" customWidth="1"/>
-    <col min="6" max="6" width="3.83203125" customWidth="1"/>
-    <col min="7" max="10" width="14.6640625" customWidth="1"/>
-    <col min="11" max="11" width="3.83203125" customWidth="1"/>
-    <col min="12" max="15" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="24.7109375" customWidth="1"/>
+    <col min="2" max="13" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:13">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="7"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="9" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="8" t="s">
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="8"/>
-      <c r="J3" s="8"/>
-      <c r="K3" s="6"/>
-      <c r="L3" s="8" t="s">
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="M3" s="8"/>
-      <c r="N3" s="8"/>
-      <c r="O3" s="8"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="9"/>
-      <c r="B4" s="1" t="s">
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="1" t="s">
+      <c r="F4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="G4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="H4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="J4" s="1" t="s">
+      <c r="I4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="6"/>
-      <c r="L4" s="1" t="s">
+      <c r="J4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="K4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="1" t="s">
+      <c r="L4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="M4" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
+    <row r="5" spans="1:13">
+      <c r="A5" s="3">
         <v>2100</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:13">
+      <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E6" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4" t="s">
+      <c r="F6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="G6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="H6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="I6" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4" t="s">
+      <c r="J6" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="K6" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="N6" s="4" t="s">
+      <c r="L6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="O6" s="4" t="s">
+      <c r="M6" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:13">
+      <c r="A7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4" t="s">
+      <c r="F7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="G7" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="H7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="I7" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4" t="s">
+      <c r="J7" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="K7" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="N7" s="4" t="s">
+      <c r="L7" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="O7" s="4" t="s">
+      <c r="M7" s="5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:13">
+      <c r="A8" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="E8" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4" t="s">
+      <c r="F8" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="G8" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="I8" s="4" t="s">
+      <c r="H8" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="I8" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="K8" s="4"/>
-      <c r="L8" s="4" t="s">
+      <c r="J8" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="K8" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="N8" s="4" t="s">
+      <c r="L8" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="O8" s="4" t="s">
+      <c r="M8" s="5" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:13">
+      <c r="A9" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4" t="s">
+      <c r="F9" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="G9" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="H9" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="I9" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="K9" s="4"/>
-      <c r="L9" s="4" t="s">
+      <c r="J9" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="K9" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="N9" s="4" t="s">
+      <c r="L9" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="O9" s="4" t="s">
+      <c r="M9" s="5" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+    <row r="10" spans="1:13">
+      <c r="A10" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="E10" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4" t="s">
+      <c r="F10" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="G10" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="H10" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="I10" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="K10" s="4"/>
-      <c r="L10" s="4" t="s">
+      <c r="J10" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="K10" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="N10" s="4" t="s">
+      <c r="L10" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="O10" s="4" t="s">
+      <c r="M10" s="5" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="2">
+    <row r="11" spans="1:13">
+      <c r="A11" s="3">
         <v>2200</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+    <row r="12" spans="1:13">
+      <c r="A12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="E12" s="4" t="s">
+      <c r="E12" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4" t="s">
+      <c r="F12" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="H12" s="4" t="s">
+      <c r="G12" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="H12" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="I12" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="K12" s="4"/>
-      <c r="L12" s="4" t="s">
+      <c r="J12" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="M12" s="4" t="s">
+      <c r="K12" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="N12" s="4" t="s">
+      <c r="L12" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="O12" s="4" t="s">
+      <c r="M12" s="5" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+    <row r="13" spans="1:13">
+      <c r="A13" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4" t="s">
+      <c r="F13" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="H13" s="4" t="s">
+      <c r="G13" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="H13" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="J13" s="4" t="s">
+      <c r="I13" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="4"/>
-      <c r="L13" s="4" t="s">
+      <c r="J13" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="M13" s="4" t="s">
+      <c r="K13" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="N13" s="4" t="s">
+      <c r="L13" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="O13" s="4" t="s">
+      <c r="M13" s="5" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:13">
+      <c r="A14" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4" t="s">
+      <c r="F14" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="G14" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="H14" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="I14" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="K14" s="4"/>
-      <c r="L14" s="4" t="s">
+      <c r="J14" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="M14" s="4" t="s">
+      <c r="K14" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="N14" s="4" t="s">
+      <c r="L14" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="O14" s="4" t="s">
+      <c r="M14" s="5" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:13">
+      <c r="A15" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="E15" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4" t="s">
+      <c r="F15" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="H15" s="4" t="s">
+      <c r="G15" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="I15" s="4" t="s">
+      <c r="H15" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="J15" s="4" t="s">
+      <c r="I15" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4" t="s">
+      <c r="J15" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="M15" s="4" t="s">
+      <c r="K15" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="N15" s="4" t="s">
+      <c r="L15" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="O15" s="4" t="s">
+      <c r="M15" s="5" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:13">
+      <c r="A16" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4" t="s">
+      <c r="F16" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="H16" s="4" t="s">
+      <c r="G16" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="I16" s="4" t="s">
+      <c r="H16" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="I16" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4" t="s">
+      <c r="J16" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="M16" s="4" t="s">
+      <c r="K16" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="N16" s="4" t="s">
+      <c r="L16" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="O16" s="4" t="s">
+      <c r="M16" s="5" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="2">
+    <row r="17" spans="1:13">
+      <c r="A17" s="3">
         <v>2300</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:13">
+      <c r="A18" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="4" t="s">
+      <c r="B18" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="E18" s="4" t="s">
+      <c r="E18" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4" t="s">
+      <c r="F18" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="H18" s="4" t="s">
+      <c r="G18" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="H18" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="I18" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4" t="s">
+      <c r="J18" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="M18" s="4" t="s">
+      <c r="K18" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="N18" s="4" t="s">
+      <c r="L18" s="5" t="s">
         <v>144</v>
       </c>
-      <c r="O18" s="4" t="s">
+      <c r="M18" s="5" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:13">
+      <c r="A19" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="E19" s="4" t="s">
+      <c r="E19" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4" t="s">
+      <c r="F19" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="H19" s="4" t="s">
+      <c r="G19" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="I19" s="4" t="s">
+      <c r="H19" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="I19" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4" t="s">
+      <c r="J19" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="M19" s="4" t="s">
+      <c r="K19" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="N19" s="4" t="s">
+      <c r="L19" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="O19" s="4" t="s">
+      <c r="M19" s="5" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
+    <row r="20" spans="1:13">
+      <c r="A20" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C20" s="4" t="s">
+      <c r="C20" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E20" s="4" t="s">
+      <c r="E20" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4" t="s">
+      <c r="F20" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="H20" s="4" t="s">
+      <c r="G20" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="H20" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="J20" s="4" t="s">
+      <c r="I20" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4" t="s">
+      <c r="J20" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="M20" s="4" t="s">
+      <c r="K20" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="N20" s="4" t="s">
+      <c r="L20" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="O20" s="4" t="s">
+      <c r="M20" s="5" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
+    <row r="21" spans="1:13">
+      <c r="A21" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="E21" s="4" t="s">
+      <c r="E21" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4" t="s">
+      <c r="F21" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="H21" s="4" t="s">
+      <c r="G21" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="I21" s="4" t="s">
+      <c r="H21" s="5" t="s">
         <v>176</v>
       </c>
-      <c r="J21" s="4" t="s">
+      <c r="I21" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4" t="s">
+      <c r="J21" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="M21" s="4" t="s">
+      <c r="K21" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="N21" s="4" t="s">
+      <c r="L21" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="O21" s="4" t="s">
+      <c r="M21" s="5" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
+    <row r="22" spans="1:13">
+      <c r="A22" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="B22" s="4" t="s">
+      <c r="B22" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="E22" s="4" t="s">
+      <c r="E22" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4" t="s">
+      <c r="F22" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="H22" s="4" t="s">
+      <c r="G22" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="H22" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="J22" s="4" t="s">
+      <c r="I22" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4" t="s">
+      <c r="J22" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="M22" s="4" t="s">
+      <c r="K22" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="N22" s="4" t="s">
+      <c r="L22" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="O22" s="4" t="s">
+      <c r="M22" s="5" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A23" s="5"/>
-      <c r="B23" s="5"/>
-      <c r="C23" s="5"/>
-      <c r="D23" s="5"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-      <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
+    <row r="23" spans="1:13">
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
+      <c r="K23" s="6"/>
+      <c r="L23" s="6"/>
+      <c r="M23" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:M1"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:E3"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="L3:O3"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="J3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup scale="55" orientation="landscape" horizontalDpi="0" verticalDpi="0"/>
+  <pageSetup fitToHeight="0" orientation="landscape"/>
 </worksheet>
 </file>
</xml_diff>